<commit_message>
# adding news and research
</commit_message>
<xml_diff>
--- a/data/cv.xlsx
+++ b/data/cv.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Library/Mobile Documents/com~apple~CloudDocs/Github/website/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED1787D-8773-3E47-ABD1-FC24070A0D10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{165EFB00-51CF-3E46-AE8C-608BC3C6BDE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="31900" windowHeight="31340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="31900" windowHeight="19120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pubs" sheetId="1" r:id="rId1"/>

</xml_diff>